<commit_message>
Added new Excel files for isentropic relations, normal shock calculations, and quasi-1D flow analysis. Updated the CompressibilityEffects.xlsx file with additional data and corrections.
</commit_message>
<xml_diff>
--- a/CompressibilityEffects.xlsx
+++ b/CompressibilityEffects.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Academics\Sem 7\Adv Gas Dynamics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{11A6F634-76DA-4604-8C99-C66392AEF7EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA9BD82-BBE5-4B8C-9727-8457898E3D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{94A6E935-1DA6-437E-80B6-6D994208DFF0}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet3 (2)" sheetId="4" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="1 per change in density" sheetId="1" r:id="rId1"/>
+    <sheet name="1 percent change in velocity" sheetId="4" r:id="rId2"/>
+    <sheet name="6 percent change in velocity" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -132,10 +132,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="8.6775371828521436E-2"/>
-          <c:y val="0.17171296296296298"/>
-          <c:w val="0.8680719597550306"/>
-          <c:h val="0.72088764946048411"/>
+          <c:x val="0.15430945348051667"/>
+          <c:y val="9.343827491489419E-2"/>
+          <c:w val="0.81445166750656839"/>
+          <c:h val="0.79916260398112371"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -170,7 +170,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$20</c:f>
+              <c:f>'1 per change in density'!$A$2:$A$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -236,7 +236,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$E$2:$E$20</c:f>
+              <c:f>'1 per change in density'!$E$2:$E$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -339,6 +339,65 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-IN"/>
+                  <a:t>Mach</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-IN" baseline="0"/>
+                  <a:t> Number</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -401,6 +460,66 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-IN"/>
+                  <a:t>Percentage</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-IN" baseline="0"/>
+                  <a:t> change in u</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-IN"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -445,7 +564,9 @@
       <c:spPr>
         <a:noFill/>
         <a:ln>
-          <a:noFill/>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
         </a:ln>
         <a:effectLst/>
       </c:spPr>
@@ -467,10 +588,7 @@
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
+        <a:schemeClr val="tx1"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -508,37 +626,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
+    <c:autoTitleDeleted val="1"/>
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
@@ -573,7 +661,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet3 (2)'!$A$2:$A$14</c:f>
+              <c:f>'1 percent change in velocity'!$A$2:$A$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
@@ -621,7 +709,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet3 (2)'!$E$2:$E$14</c:f>
+              <c:f>'1 percent change in velocity'!$E$2:$E$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
@@ -703,7 +791,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet3 (2)'!$A$15:$A$20</c:f>
+              <c:f>'1 percent change in velocity'!$A$15:$A$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -730,7 +818,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet3 (2)'!$E$15:$E$20</c:f>
+              <c:f>'1 percent change in velocity'!$E$15:$E$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -794,6 +882,61 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-IN"/>
+                  <a:t>Mach Number</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -856,6 +999,66 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-IN"/>
+                  <a:t>Percentage</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-IN" baseline="0"/>
+                  <a:t> change in density</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-IN"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -922,10 +1125,7 @@
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
+        <a:schemeClr val="tx1"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -964,6 +1164,36 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-IN"/>
+              <a:t>&lt;</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-IN" baseline="0"/>
+              <a:t> M = 1</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-IN"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -972,26 +1202,6 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -1004,7 +1214,7 @@
           <c:order val="0"/>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet3!$A$2:$A$14</c:f>
+              <c:f>'6 percent change in velocity'!$A$2:$A$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
@@ -1052,7 +1262,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet3!$E$2:$E$14</c:f>
+              <c:f>'6 percent change in velocity'!$E$2:$E$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
@@ -1137,6 +1347,24 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-IN"/>
+                  <a:t>Mach Number</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1199,6 +1427,36 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-IN"/>
+                  <a:t>Percentage</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-IN" baseline="0"/>
+                  <a:t> change in density</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="1.9372535926453643E-2"/>
+              <c:y val="0.32206126987353823"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1246,6 +1504,13 @@
     <c:showDLblsOverMax val="0"/>
     <c:extLst/>
   </c:chart>
+  <c:spPr>
+    <a:ln>
+      <a:solidFill>
+        <a:schemeClr val="tx1"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
   <c:txPr>
     <a:bodyPr/>
     <a:lstStyle/>
@@ -1279,6 +1544,35 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-IN"/>
+              <a:t>&gt;=</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-IN" baseline="0"/>
+              <a:t> M = 1</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1343,7 +1637,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet3!$A$15:$A$20</c:f>
+              <c:f>'6 percent change in velocity'!$A$15:$A$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1370,7 +1664,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet3!$E$15:$E$20</c:f>
+              <c:f>'6 percent change in velocity'!$E$15:$E$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1434,6 +1728,65 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-IN"/>
+                  <a:t>Mach</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-IN" baseline="0"/>
+                  <a:t> Number</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1496,6 +1849,66 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-IN"/>
+                  <a:t>Percentage</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-IN" baseline="0"/>
+                  <a:t> Change in density</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-IN"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1562,10 +1975,7 @@
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
+        <a:schemeClr val="tx1"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -3261,16 +3671,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>83820</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>448654</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>388620</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>26670</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>534112</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>56972</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3302,16 +3712,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>34290</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>409755</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>34290</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>323491</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3346,15 +3756,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>469725</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>100209</xdr:rowOff>
+      <xdr:colOff>552551</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>198328</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>25053</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>124239</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>24847</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3382,15 +3792,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>516194</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>136016</xdr:rowOff>
+      <xdr:colOff>541041</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>127733</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>237613</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>175345</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>124239</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>49694</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4118,7 +4528,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
         <v>4</v>

</xml_diff>